<commit_message>
correct ^ for ** in calc; minor change CHartJS adapter
</commit_message>
<xml_diff>
--- a/test/Bioreactor_forPy.xlsx
+++ b/test/Bioreactor_forPy.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Server\Tools\python\FermentALADIN\FermentationModel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Server\Tools\python\FermentALADIN\FermentationModel\test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12F19D8B-B417-450B-A490-2A959DE60903}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B137A29-417E-4F57-8CBB-E8FFFBB61A62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{66E3D132-4FA8-40D7-B6AE-50FDCDDD87B9}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="24892" windowHeight="14914" activeTab="1" xr2:uid="{66E3D132-4FA8-40D7-B6AE-50FDCDDD87B9}"/>
   </bookViews>
   <sheets>
     <sheet name="Hübsch" sheetId="5" r:id="rId1"/>
@@ -2344,13 +2344,17 @@
         <v>40</v>
       </c>
       <c r="N3" s="39">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="O3" s="61">
-        <v>20</v>
-      </c>
-      <c r="P3" s="62"/>
-      <c r="Q3" s="39"/>
+        <v>0</v>
+      </c>
+      <c r="P3" s="62">
+        <v>0</v>
+      </c>
+      <c r="Q3" s="39">
+        <v>0</v>
+      </c>
       <c r="R3" s="29"/>
       <c r="S3" s="28"/>
       <c r="T3" s="28"/>
@@ -2427,7 +2431,7 @@
       <c r="N5" s="30"/>
       <c r="O5" s="34">
         <f>SUM(N3:Q3)</f>
-        <v>40</v>
+        <v>12</v>
       </c>
       <c r="P5" s="34" t="s">
         <v>17</v>
@@ -2460,7 +2464,7 @@
         <v>0</v>
       </c>
       <c r="G6" s="37">
-        <v>500</v>
+        <v>800</v>
       </c>
       <c r="H6" s="40"/>
       <c r="K6" s="40"/>
@@ -2489,19 +2493,15 @@
       <c r="B7" s="40"/>
       <c r="C7" s="15">
         <f>C6+$N$3</f>
-        <v>20</v>
-      </c>
-      <c r="D7" s="37">
-        <v>0.2</v>
-      </c>
+        <v>12</v>
+      </c>
+      <c r="D7" s="37"/>
       <c r="E7" s="40"/>
       <c r="F7" s="15">
         <f>F6+$N$3</f>
-        <v>20</v>
-      </c>
-      <c r="G7" s="37">
-        <v>1000</v>
-      </c>
+        <v>12</v>
+      </c>
+      <c r="G7" s="37"/>
       <c r="H7" s="40"/>
       <c r="I7" s="40"/>
       <c r="J7" s="40"/>
@@ -2531,13 +2531,13 @@
       <c r="B8" s="40"/>
       <c r="C8" s="15">
         <f>C7+$O$3</f>
-        <v>40</v>
+        <v>12</v>
       </c>
       <c r="D8" s="37"/>
       <c r="E8" s="40"/>
       <c r="F8" s="15">
         <f>F7+$O$3</f>
-        <v>40</v>
+        <v>12</v>
       </c>
       <c r="G8" s="37"/>
       <c r="H8" s="40"/>
@@ -2569,13 +2569,13 @@
       <c r="B9" s="40"/>
       <c r="C9" s="15">
         <f>C8+$P$3</f>
-        <v>40</v>
+        <v>12</v>
       </c>
       <c r="D9" s="37"/>
       <c r="E9" s="40"/>
       <c r="F9" s="15">
         <f>F8+$P$3</f>
-        <v>40</v>
+        <v>12</v>
       </c>
       <c r="G9" s="37"/>
       <c r="H9" s="40"/>
@@ -2763,7 +2763,7 @@
         <v>0</v>
       </c>
       <c r="Q14" s="37">
-        <v>5</v>
+        <v>100</v>
       </c>
       <c r="R14" s="37"/>
       <c r="S14" s="40"/>
@@ -2786,7 +2786,7 @@
         <v>0</v>
       </c>
       <c r="D15" s="37">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="E15" s="40"/>
       <c r="F15" s="5"/>
@@ -2811,12 +2811,10 @@
       <c r="O15" s="40"/>
       <c r="P15" s="15">
         <f>P14+$N$3</f>
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="Q15" s="37"/>
-      <c r="R15" s="37">
-        <v>4</v>
-      </c>
+      <c r="R15" s="37"/>
       <c r="S15" s="40"/>
       <c r="T15" s="40"/>
       <c r="U15" s="28"/>
@@ -2835,11 +2833,9 @@
       <c r="B16" s="40"/>
       <c r="C16" s="15">
         <f>C15+$N$3</f>
-        <v>20</v>
-      </c>
-      <c r="D16" s="37">
-        <v>100</v>
-      </c>
+        <v>12</v>
+      </c>
+      <c r="D16" s="37"/>
       <c r="E16" s="40"/>
       <c r="F16" s="5"/>
       <c r="G16" s="12">
@@ -2864,7 +2860,7 @@
       <c r="O16" s="40"/>
       <c r="P16" s="15">
         <f>P15+$O$3</f>
-        <v>40</v>
+        <v>12</v>
       </c>
       <c r="Q16" s="37"/>
       <c r="R16" s="37"/>
@@ -2886,7 +2882,7 @@
       <c r="B17" s="40"/>
       <c r="C17" s="15">
         <f>C16+$O$3</f>
-        <v>40</v>
+        <v>12</v>
       </c>
       <c r="D17" s="37"/>
       <c r="E17" s="40"/>
@@ -2904,7 +2900,7 @@
       <c r="O17" s="40"/>
       <c r="P17" s="15">
         <f>P16+$P$3</f>
-        <v>40</v>
+        <v>12</v>
       </c>
       <c r="Q17" s="38"/>
       <c r="R17" s="37"/>
@@ -2926,7 +2922,7 @@
       <c r="B18" s="40"/>
       <c r="C18" s="15">
         <f>C17+$P$3</f>
-        <v>40</v>
+        <v>12</v>
       </c>
       <c r="D18" s="37"/>
       <c r="E18" s="40"/>
@@ -2949,11 +2945,11 @@
       </c>
       <c r="Q18" s="50">
         <f>SUM(Q14:Q17)</f>
-        <v>5</v>
+        <v>100</v>
       </c>
       <c r="R18" s="51">
         <f>SUMPRODUCT(Input_Array!D4:D7,Input_Array!H4:H7)</f>
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="S18" s="42"/>
       <c r="T18" s="42"/>
@@ -2976,7 +2972,7 @@
       <c r="E19" s="40"/>
       <c r="F19" s="5"/>
       <c r="G19" s="54">
-        <v>100</v>
+        <v>20</v>
       </c>
       <c r="H19" s="10" t="s">
         <v>23</v>
@@ -3062,7 +3058,7 @@
         <v>37</v>
       </c>
       <c r="L21" s="55">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="M21" s="13" t="s">
         <v>9</v>
@@ -3158,11 +3154,9 @@
       <c r="O23" s="40"/>
       <c r="P23" s="15">
         <f>P22+$N$3</f>
-        <v>20</v>
-      </c>
-      <c r="Q23" s="37">
-        <v>10</v>
-      </c>
+        <v>12</v>
+      </c>
+      <c r="Q23" s="37"/>
       <c r="R23" s="28"/>
       <c r="S23" s="40"/>
       <c r="T23" s="40"/>
@@ -3196,7 +3190,7 @@
       <c r="O24" s="40"/>
       <c r="P24" s="15">
         <f>P23+$O$3</f>
-        <v>40</v>
+        <v>12</v>
       </c>
       <c r="Q24" s="37"/>
       <c r="R24" s="28"/>
@@ -3233,7 +3227,7 @@
       <c r="O25" s="40"/>
       <c r="P25" s="53">
         <f>P24+$P$3</f>
-        <v>40</v>
+        <v>12</v>
       </c>
       <c r="Q25" s="38"/>
       <c r="R25" s="28"/>
@@ -3273,7 +3267,7 @@
       </c>
       <c r="Q26" s="50">
         <f>SUM(Q22:Q25)</f>
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="R26" s="28"/>
       <c r="S26" s="40"/>
@@ -3779,11 +3773,11 @@
       </c>
       <c r="B4">
         <f>Hübsch!D15</f>
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="C4" cm="1">
         <f t="array" ref="C4:C7">Hübsch!Q14:Q17</f>
-        <v>5</v>
+        <v>100</v>
       </c>
       <c r="D4">
         <f>Hübsch!R14</f>
@@ -3795,7 +3789,7 @@
       </c>
       <c r="F4">
         <f>Hübsch!G6</f>
-        <v>500</v>
+        <v>800</v>
       </c>
       <c r="G4">
         <f>Hübsch!D6</f>
@@ -3803,11 +3797,11 @@
       </c>
       <c r="H4">
         <f>Hübsch!N3</f>
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="I4">
         <f>Hübsch!$G$19</f>
-        <v>100</v>
+        <v>20</v>
       </c>
       <c r="J4">
         <f>Hübsch!$L$15</f>
@@ -3823,7 +3817,7 @@
       </c>
       <c r="N4">
         <f>Hübsch!L21</f>
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="O4">
         <v>0</v>
@@ -3839,34 +3833,34 @@
       </c>
       <c r="B5">
         <f>Hübsch!D16</f>
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="C5">
         <v>0</v>
       </c>
       <c r="D5">
         <f>Hübsch!R15</f>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E5">
         <f>Hübsch!Q23</f>
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="F5">
         <f>Hübsch!G7</f>
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="G5">
         <f>Hübsch!D7</f>
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="H5">
         <f>Hübsch!O3</f>
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="I5">
         <f>Hübsch!$G$19</f>
-        <v>100</v>
+        <v>20</v>
       </c>
       <c r="J5">
         <f>Hübsch!$L$15</f>
@@ -3916,7 +3910,7 @@
       </c>
       <c r="I6">
         <f>Hübsch!$G$19</f>
-        <v>100</v>
+        <v>20</v>
       </c>
       <c r="J6">
         <f>Hübsch!$L$15</f>
@@ -3966,7 +3960,7 @@
       </c>
       <c r="I7">
         <f>Hübsch!$G$19</f>
-        <v>100</v>
+        <v>20</v>
       </c>
       <c r="J7">
         <f>Hübsch!$L$15</f>

</xml_diff>